<commit_message>
Phase 4: executive dashboard
- Greeting by time of day + since-last-login line
- Portfolio Intelligence: generated brief (occupancy/revenue, money at
  risk, renewals, weakest building, vacancy) with three "Today" moves —
  recomputed from queries on every change
- 4 hero KPIs with month-over-month trends + quiet strip
- Needs attention (top 5 critical, inline actions), Next 30 days
  (expiring contracts + payments due), revenue chart (collected bars,
  billed line, table view, CVD-validated palette), property ranking with
  occupancy/revenue/outstanding/score and portfolio total row, vacancy
  opportunity card
- ActionsProvider: one dispatcher for alert actions and write flows
- Reliable = full year never late; seed makes Nadine the sole reliable
  renewal

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/seed/cedar-residence.xlsx
+++ b/public/seed/cedar-residence.xlsx
@@ -696,16 +696,16 @@
         <v>2</v>
       </c>
       <c r="F2">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="G2" t="str">
         <v>no</v>
       </c>
       <c r="H2">
-        <v>1075</v>
+        <v>1125</v>
       </c>
       <c r="I2">
-        <v>1075</v>
+        <v>1125</v>
       </c>
       <c r="J2" t="str">
         <v/>
@@ -731,16 +731,16 @@
         <v>1</v>
       </c>
       <c r="F3">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G3" t="str">
         <v>no</v>
       </c>
       <c r="H3">
-        <v>900</v>
+        <v>975</v>
       </c>
       <c r="I3">
-        <v>900</v>
+        <v>975</v>
       </c>
       <c r="J3" t="str">
         <v/>
@@ -766,16 +766,16 @@
         <v>1</v>
       </c>
       <c r="F4">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="G4" t="str">
-        <v>no</v>
+        <v>yes</v>
       </c>
       <c r="H4">
-        <v>800</v>
+        <v>775</v>
       </c>
       <c r="I4">
-        <v>800</v>
+        <v>775</v>
       </c>
       <c r="J4" t="str">
         <v/>
@@ -801,16 +801,16 @@
         <v>2</v>
       </c>
       <c r="F5">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G5" t="str">
-        <v>yes</v>
+        <v>no</v>
       </c>
       <c r="H5">
-        <v>1200</v>
+        <v>1150</v>
       </c>
       <c r="I5">
-        <v>1200</v>
+        <v>1150</v>
       </c>
       <c r="J5" t="str">
         <v/>
@@ -836,16 +836,16 @@
         <v>1</v>
       </c>
       <c r="F6">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G6" t="str">
-        <v>no</v>
+        <v>yes</v>
       </c>
       <c r="H6">
-        <v>925</v>
+        <v>1000</v>
       </c>
       <c r="I6">
-        <v>925</v>
+        <v>1000</v>
       </c>
       <c r="J6" t="str">
         <v/>
@@ -871,16 +871,16 @@
         <v>1</v>
       </c>
       <c r="F7">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="G7" t="str">
         <v>no</v>
       </c>
       <c r="H7">
-        <v>775</v>
+        <v>800</v>
       </c>
       <c r="I7">
-        <v>775</v>
+        <v>800</v>
       </c>
       <c r="J7" t="str">
         <v/>
@@ -906,16 +906,16 @@
         <v>2</v>
       </c>
       <c r="F8">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="G8" t="str">
         <v>yes</v>
       </c>
       <c r="H8">
-        <v>1200</v>
+        <v>1175</v>
       </c>
       <c r="I8">
-        <v>1200</v>
+        <v>1175</v>
       </c>
       <c r="J8" t="str">
         <v/>
@@ -941,16 +941,16 @@
         <v>1</v>
       </c>
       <c r="F9">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="G9" t="str">
-        <v>yes</v>
+        <v>no</v>
       </c>
       <c r="H9">
-        <v>925</v>
+        <v>1025</v>
       </c>
       <c r="I9">
-        <v>925</v>
+        <v>1025</v>
       </c>
       <c r="J9" t="str">
         <v/>
@@ -976,16 +976,16 @@
         <v>1</v>
       </c>
       <c r="F10">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="G10" t="str">
         <v>yes</v>
       </c>
       <c r="H10">
-        <v>775</v>
+        <v>825</v>
       </c>
       <c r="I10">
-        <v>775</v>
+        <v>825</v>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -1011,16 +1011,16 @@
         <v>2</v>
       </c>
       <c r="F11">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G11" t="str">
-        <v>no</v>
+        <v>yes</v>
       </c>
       <c r="H11">
-        <v>1125</v>
+        <v>1250</v>
       </c>
       <c r="I11">
-        <v>1125</v>
+        <v>1250</v>
       </c>
       <c r="J11" t="str">
         <v/>
@@ -1046,16 +1046,16 @@
         <v>1</v>
       </c>
       <c r="F12">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="G12" t="str">
         <v>no</v>
       </c>
       <c r="H12">
-        <v>1000</v>
+        <v>1050</v>
       </c>
       <c r="I12">
-        <v>1000</v>
+        <v>1050</v>
       </c>
       <c r="J12" t="str">
         <v/>
@@ -1081,16 +1081,16 @@
         <v>1</v>
       </c>
       <c r="F13">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="G13" t="str">
         <v>no</v>
       </c>
       <c r="H13">
-        <v>800</v>
+        <v>900</v>
       </c>
       <c r="I13">
-        <v>800</v>
+        <v>900</v>
       </c>
       <c r="J13" t="str">
         <v/>
@@ -1116,16 +1116,16 @@
         <v>2</v>
       </c>
       <c r="F14">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="G14" t="str">
         <v>no</v>
       </c>
       <c r="H14">
-        <v>1250</v>
+        <v>1150</v>
       </c>
       <c r="I14">
-        <v>1250</v>
+        <v>1150</v>
       </c>
       <c r="J14" t="str">
         <v/>
@@ -1151,7 +1151,7 @@
         <v>1</v>
       </c>
       <c r="F15">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G15" t="str">
         <v>no</v>
@@ -1186,16 +1186,16 @@
         <v>1</v>
       </c>
       <c r="F16">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="G16" t="str">
         <v>no</v>
       </c>
       <c r="H16">
-        <v>825</v>
+        <v>875</v>
       </c>
       <c r="I16">
-        <v>825</v>
+        <v>875</v>
       </c>
       <c r="J16" t="str">
         <v/>
@@ -1221,16 +1221,16 @@
         <v>2</v>
       </c>
       <c r="F17">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="G17" t="str">
-        <v>no</v>
+        <v>yes</v>
       </c>
       <c r="H17">
-        <v>1200</v>
+        <v>1275</v>
       </c>
       <c r="I17">
-        <v>1200</v>
+        <v>1275</v>
       </c>
       <c r="J17" t="str">
         <v/>
@@ -1256,16 +1256,16 @@
         <v>1</v>
       </c>
       <c r="F18">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="G18" t="str">
         <v>no</v>
       </c>
       <c r="H18">
-        <v>1050</v>
+        <v>1000</v>
       </c>
       <c r="I18">
-        <v>1050</v>
+        <v>1000</v>
       </c>
       <c r="J18" t="str">
         <v/>
@@ -1291,16 +1291,16 @@
         <v>1</v>
       </c>
       <c r="F19">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="G19" t="str">
-        <v>yes</v>
+        <v>no</v>
       </c>
       <c r="H19">
-        <v>900</v>
+        <v>850</v>
       </c>
       <c r="I19">
-        <v>900</v>
+        <v>850</v>
       </c>
       <c r="J19" t="str">
         <v/>
@@ -1370,34 +1370,34 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Marie</v>
+        <v>Jad</v>
       </c>
       <c r="B2" t="str">
-        <v>Rizk</v>
+        <v>Dagher</v>
       </c>
       <c r="C2" t="str">
-        <v>+961 81 170 216</v>
+        <v>+961 70 489 845</v>
       </c>
       <c r="D2" t="str">
-        <v>marie.rizk@example.com</v>
+        <v>jad.dagher@example.com</v>
       </c>
       <c r="E2" t="str">
         <v>Lebanese</v>
       </c>
       <c r="F2" t="str">
-        <v>passport</v>
+        <v>national_id</v>
       </c>
       <c r="G2" t="str">
-        <v>RL6979454</v>
+        <v>LB-6900604</v>
       </c>
       <c r="H2" t="str">
-        <v>Accountant</v>
+        <v>Designer</v>
       </c>
       <c r="I2" t="str">
-        <v>Rafic Rizk</v>
+        <v/>
       </c>
       <c r="J2" t="str">
-        <v/>
+        <v>+961 71 534 988</v>
       </c>
       <c r="K2" t="str">
         <v/>
@@ -1405,16 +1405,16 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Nabil</v>
+        <v>Rima</v>
       </c>
       <c r="B3" t="str">
-        <v>Osseiran</v>
+        <v>Fares</v>
       </c>
       <c r="C3" t="str">
-        <v>+961 71 235 156</v>
+        <v>+961 78 642 109</v>
       </c>
       <c r="D3" t="str">
-        <v>nabil.osseiran@example.com</v>
+        <v>rima.fares@example.com</v>
       </c>
       <c r="E3" t="str">
         <v>Lebanese</v>
@@ -1423,16 +1423,16 @@
         <v>national_id</v>
       </c>
       <c r="G3" t="str">
-        <v>LB-8914569</v>
+        <v>LB-1685442</v>
       </c>
       <c r="H3" t="str">
-        <v>Designer</v>
+        <v>Bank officer</v>
       </c>
       <c r="I3" t="str">
-        <v>Dima Osseiran</v>
+        <v/>
       </c>
       <c r="J3" t="str">
-        <v>+961 3 759 930</v>
+        <v>+961 79 751 636</v>
       </c>
       <c r="K3" t="str">
         <v/>
@@ -1440,16 +1440,16 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Sandra</v>
+        <v>Antoine</v>
       </c>
       <c r="B4" t="str">
-        <v>Hajj</v>
+        <v>Baydoun</v>
       </c>
       <c r="C4" t="str">
-        <v>+961 70 361 683</v>
+        <v>+961 70 108 759</v>
       </c>
       <c r="D4" t="str">
-        <v>sandra.hajj@example.com</v>
+        <v>antoine.baydoun@example.com</v>
       </c>
       <c r="E4" t="str">
         <v>Lebanese</v>
@@ -1458,16 +1458,16 @@
         <v>national_id</v>
       </c>
       <c r="G4" t="str">
-        <v/>
+        <v>LB-7737871</v>
       </c>
       <c r="H4" t="str">
-        <v>Consultant</v>
+        <v>Journalist</v>
       </c>
       <c r="I4" t="str">
-        <v>Salim Hajj</v>
+        <v/>
       </c>
       <c r="J4" t="str">
-        <v>+961 71 947 538</v>
+        <v>+961 76 953 284</v>
       </c>
       <c r="K4" t="str">
         <v/>
@@ -1475,16 +1475,16 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Maria</v>
+        <v>Antoine</v>
       </c>
       <c r="B5" t="str">
-        <v>Chehab</v>
+        <v>Nasrallah</v>
       </c>
       <c r="C5" t="str">
-        <v>+961 78 442 534</v>
+        <v>+961 78 258 933</v>
       </c>
       <c r="D5" t="str">
-        <v>maria.chehab@example.com</v>
+        <v>antoine.nasrallah@example.com</v>
       </c>
       <c r="E5" t="str">
         <v>Lebanese</v>
@@ -1493,16 +1493,16 @@
         <v>national_id</v>
       </c>
       <c r="G5" t="str">
-        <v>LB-2236731</v>
+        <v>LB-4126818</v>
       </c>
       <c r="H5" t="str">
-        <v>Engineer</v>
+        <v>Bank officer</v>
       </c>
       <c r="I5" t="str">
-        <v/>
+        <v>Nada Nasrallah</v>
       </c>
       <c r="J5" t="str">
-        <v>+961 76 570 797</v>
+        <v>+961 79 386 582</v>
       </c>
       <c r="K5" t="str">
         <v/>
@@ -1510,34 +1510,34 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Tamara</v>
+        <v>Rony</v>
       </c>
       <c r="B6" t="str">
-        <v>Nakhle</v>
+        <v>Hajj</v>
       </c>
       <c r="C6" t="str">
-        <v>+961 70 219 593</v>
+        <v>+961 81 751 494</v>
       </c>
       <c r="D6" t="str">
-        <v>tamara.nakhle@example.com</v>
+        <v>rony.hajj@example.com</v>
       </c>
       <c r="E6" t="str">
-        <v>Lebanese</v>
+        <v>Jordanian</v>
       </c>
       <c r="F6" t="str">
-        <v>national_id</v>
+        <v>passport</v>
       </c>
       <c r="G6" t="str">
-        <v>LB-8270749</v>
+        <v>RL4787623</v>
       </c>
       <c r="H6" t="str">
         <v>Bank officer</v>
       </c>
       <c r="I6" t="str">
-        <v>Fouad Nakhle</v>
+        <v/>
       </c>
       <c r="J6" t="str">
-        <v/>
+        <v>+961 76 784 663</v>
       </c>
       <c r="K6" t="str">
         <v/>
@@ -1545,34 +1545,34 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Jessica</v>
+        <v>Maya</v>
       </c>
       <c r="B7" t="str">
-        <v>Makhlouf</v>
+        <v>Rizk</v>
       </c>
       <c r="C7" t="str">
-        <v>+961 81 284 501</v>
+        <v>+961 79 533 713</v>
       </c>
       <c r="D7" t="str">
-        <v>jessica.makhlouf@example.com</v>
+        <v>maya.rizk@example.com</v>
       </c>
       <c r="E7" t="str">
-        <v>Syrian</v>
+        <v>Egyptian</v>
       </c>
       <c r="F7" t="str">
         <v>passport</v>
       </c>
       <c r="G7" t="str">
-        <v>RL9994819</v>
+        <v>RL6775325</v>
       </c>
       <c r="H7" t="str">
-        <v>Nurse</v>
+        <v>Accountant</v>
       </c>
       <c r="I7" t="str">
-        <v/>
+        <v>Khaled Rizk</v>
       </c>
       <c r="J7" t="str">
-        <v>+961 81 334 111</v>
+        <v/>
       </c>
       <c r="K7" t="str">
         <v/>
@@ -1580,34 +1580,34 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Nicolas</v>
+        <v>Roy</v>
       </c>
       <c r="B8" t="str">
-        <v>Hobeika</v>
+        <v>Fakhoury</v>
       </c>
       <c r="C8" t="str">
-        <v>+961 78 477 783</v>
+        <v>+961 71 801 321</v>
       </c>
       <c r="D8" t="str">
-        <v>nicolas.hobeika@example.com</v>
+        <v>roy.fakhoury@example.com</v>
       </c>
       <c r="E8" t="str">
         <v>Lebanese</v>
       </c>
       <c r="F8" t="str">
-        <v>national_id</v>
+        <v>passport</v>
       </c>
       <c r="G8" t="str">
-        <v>LB-5823991</v>
+        <v>RL4085610</v>
       </c>
       <c r="H8" t="str">
-        <v>Consultant</v>
+        <v>Designer</v>
       </c>
       <c r="I8" t="str">
-        <v/>
+        <v>Marie Fakhoury</v>
       </c>
       <c r="J8" t="str">
-        <v/>
+        <v>+961 70 164 924</v>
       </c>
       <c r="K8" t="str">
         <v/>
@@ -1615,31 +1615,31 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Tamara</v>
+        <v>Ali</v>
       </c>
       <c r="B9" t="str">
-        <v>Kassab</v>
+        <v>Nassar</v>
       </c>
       <c r="C9" t="str">
-        <v>+961 3 478 366</v>
+        <v>+961 78 828 106</v>
       </c>
       <c r="D9" t="str">
-        <v>tamara.kassab@example.com</v>
+        <v>ali.nassar@example.com</v>
       </c>
       <c r="E9" t="str">
-        <v>Lebanese</v>
+        <v>Canadian</v>
       </c>
       <c r="F9" t="str">
-        <v>national_id</v>
+        <v>passport</v>
       </c>
       <c r="G9" t="str">
-        <v>LB-6824243</v>
+        <v>RL7106746</v>
       </c>
       <c r="H9" t="str">
-        <v>Restaurant owner</v>
+        <v>Consultant</v>
       </c>
       <c r="I9" t="str">
-        <v>Lara Kassab</v>
+        <v/>
       </c>
       <c r="J9" t="str">
         <v/>
@@ -1650,16 +1650,16 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Imad</v>
+        <v>Sandra</v>
       </c>
       <c r="B10" t="str">
-        <v>Farah</v>
+        <v>Baydoun</v>
       </c>
       <c r="C10" t="str">
-        <v>+961 78 848 533</v>
+        <v>+961 79 438 693</v>
       </c>
       <c r="D10" t="str">
-        <v>imad.farah@example.com</v>
+        <v>sandra.baydoun@example.com</v>
       </c>
       <c r="E10" t="str">
         <v>Lebanese</v>
@@ -1668,16 +1668,16 @@
         <v>national_id</v>
       </c>
       <c r="G10" t="str">
-        <v>LB-1334610</v>
+        <v>LB-6019906</v>
       </c>
       <c r="H10" t="str">
-        <v>Bank officer</v>
+        <v>Architect</v>
       </c>
       <c r="I10" t="str">
-        <v>Ghassan Farah</v>
+        <v>Kamal Baydoun</v>
       </c>
       <c r="J10" t="str">
-        <v>+961 78 279 949</v>
+        <v>+961 70 550 287</v>
       </c>
       <c r="K10" t="str">
         <v/>
@@ -1685,34 +1685,34 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Roy</v>
+        <v>Imad</v>
       </c>
       <c r="B11" t="str">
-        <v>Fakhoury</v>
+        <v>Maalouf</v>
       </c>
       <c r="C11" t="str">
-        <v>+961 71 801 321</v>
+        <v>+961 78 872 553</v>
       </c>
       <c r="D11" t="str">
-        <v>roy.fakhoury@example.com</v>
+        <v>imad.maalouf@example.com</v>
       </c>
       <c r="E11" t="str">
         <v>Lebanese</v>
       </c>
       <c r="F11" t="str">
-        <v>passport</v>
+        <v>national_id</v>
       </c>
       <c r="G11" t="str">
-        <v>RL4085610</v>
+        <v>LB-8511653</v>
       </c>
       <c r="H11" t="str">
-        <v>Designer</v>
+        <v>Teacher</v>
       </c>
       <c r="I11" t="str">
-        <v>Marie Fakhoury</v>
+        <v>Sara Maalouf</v>
       </c>
       <c r="J11" t="str">
-        <v>+961 70 164 924</v>
+        <v/>
       </c>
       <c r="K11" t="str">
         <v/>
@@ -1720,34 +1720,34 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Ali</v>
+        <v>Walid</v>
       </c>
       <c r="B12" t="str">
-        <v>Nassar</v>
+        <v>Ayoub</v>
       </c>
       <c r="C12" t="str">
-        <v>+961 78 828 106</v>
+        <v>+961 70 701 949</v>
       </c>
       <c r="D12" t="str">
-        <v>ali.nassar@example.com</v>
+        <v>walid.ayoub@example.com</v>
       </c>
       <c r="E12" t="str">
-        <v>Canadian</v>
+        <v>Syrian</v>
       </c>
       <c r="F12" t="str">
         <v>passport</v>
       </c>
       <c r="G12" t="str">
-        <v>RL7106746</v>
+        <v>RL1245733</v>
       </c>
       <c r="H12" t="str">
-        <v>Consultant</v>
+        <v>Nurse</v>
       </c>
       <c r="I12" t="str">
-        <v/>
+        <v>Rita Ayoub</v>
       </c>
       <c r="J12" t="str">
-        <v/>
+        <v>+961 78 647 728</v>
       </c>
       <c r="K12" t="str">
         <v/>
@@ -1755,34 +1755,34 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Christine</v>
+        <v>Tarek</v>
       </c>
       <c r="B13" t="str">
-        <v>Saade</v>
+        <v>Kfoury</v>
       </c>
       <c r="C13" t="str">
-        <v>+961 71 601 199</v>
+        <v>+961 81 524 789</v>
       </c>
       <c r="D13" t="str">
-        <v>christine.saade@example.com</v>
+        <v>tarek.kfoury@example.com</v>
       </c>
       <c r="E13" t="str">
         <v>Lebanese</v>
       </c>
       <c r="F13" t="str">
-        <v>national_id</v>
+        <v>passport</v>
       </c>
       <c r="G13" t="str">
-        <v>LB-3852143</v>
+        <v>RL5683314</v>
       </c>
       <c r="H13" t="str">
         <v>Bank officer</v>
       </c>
       <c r="I13" t="str">
-        <v>Nadine Saade</v>
+        <v>Pascale Kfoury</v>
       </c>
       <c r="J13" t="str">
-        <v>+961 81 711 622</v>
+        <v>+961 70 267 964</v>
       </c>
       <c r="K13" t="str">
         <v/>
@@ -1790,31 +1790,31 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Mariam</v>
+        <v>Tala</v>
       </c>
       <c r="B14" t="str">
-        <v>Makhlouf</v>
+        <v>Chehab</v>
       </c>
       <c r="C14" t="str">
-        <v>+961 76 851 237</v>
+        <v>+961 70 969 500</v>
       </c>
       <c r="D14" t="str">
-        <v>mariam.makhlouf@example.com</v>
+        <v>tala.chehab@example.com</v>
       </c>
       <c r="E14" t="str">
         <v>Lebanese</v>
       </c>
       <c r="F14" t="str">
-        <v>national_id</v>
+        <v>passport</v>
       </c>
       <c r="G14" t="str">
-        <v>LB-6790836</v>
+        <v>RL5435856</v>
       </c>
       <c r="H14" t="str">
-        <v>Sales manager</v>
+        <v>Lawyer</v>
       </c>
       <c r="I14" t="str">
-        <v>Josiane Makhlouf</v>
+        <v>Pascale Chehab</v>
       </c>
       <c r="J14" t="str">
         <v/>
@@ -1825,34 +1825,34 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Nicolas</v>
+        <v>Selim</v>
       </c>
       <c r="B15" t="str">
-        <v>Hijazi</v>
+        <v>Kassab</v>
       </c>
       <c r="C15" t="str">
-        <v>+961 70 124 242</v>
+        <v>+961 3 800 428</v>
       </c>
       <c r="D15" t="str">
-        <v>nicolas.hijazi@example.com</v>
+        <v>selim.kassab@example.com</v>
       </c>
       <c r="E15" t="str">
         <v>Lebanese</v>
       </c>
       <c r="F15" t="str">
-        <v>passport</v>
+        <v>national_id</v>
       </c>
       <c r="G15" t="str">
-        <v>RL5267604</v>
+        <v>LB-4604729</v>
       </c>
       <c r="H15" t="str">
-        <v>Designer</v>
+        <v>Physician</v>
       </c>
       <c r="I15" t="str">
-        <v>Rima Hijazi</v>
+        <v>Fadi Kassab</v>
       </c>
       <c r="J15" t="str">
-        <v>+961 78 526 749</v>
+        <v/>
       </c>
       <c r="K15" t="str">
         <v/>
@@ -1931,22 +1931,22 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>CR-103-01</v>
+        <v>CR-203-01</v>
       </c>
       <c r="B2" t="str">
         <v>CR</v>
       </c>
       <c r="C2" t="str">
-        <v>103</v>
+        <v>203</v>
       </c>
       <c r="D2" t="str">
-        <v>+961 81 170 216</v>
+        <v>+961 70 489 845</v>
       </c>
       <c r="E2" t="str">
-        <v>today+286d-12m</v>
+        <v>today+98d-24m</v>
       </c>
       <c r="F2" t="str">
-        <v>today+286d</v>
+        <v>today+98d</v>
       </c>
       <c r="G2">
         <v>800</v>
@@ -1955,10 +1955,10 @@
         <v>800</v>
       </c>
       <c r="I2">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="J2" t="str">
-        <v>cash</v>
+        <v>bank_transfer</v>
       </c>
       <c r="K2" t="str">
         <v/>
@@ -1975,34 +1975,34 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>CR-102-01</v>
+        <v>CR-103-01</v>
       </c>
       <c r="B3" t="str">
         <v>CR</v>
       </c>
       <c r="C3" t="str">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D3" t="str">
-        <v>+961 71 235 156</v>
+        <v>+961 78 642 109</v>
       </c>
       <c r="E3" t="str">
-        <v>today+187d-12m</v>
+        <v>today+130d-24m</v>
       </c>
       <c r="F3" t="str">
-        <v>today+187d</v>
+        <v>today+130d</v>
       </c>
       <c r="G3">
-        <v>900</v>
+        <v>775</v>
       </c>
       <c r="H3">
-        <v>900</v>
+        <v>775</v>
       </c>
       <c r="I3">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="J3" t="str">
-        <v>bank_transfer</v>
+        <v>cheque</v>
       </c>
       <c r="K3" t="str">
         <v/>
@@ -2019,31 +2019,31 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>CR-501-01</v>
+        <v>CR-202-01</v>
       </c>
       <c r="B4" t="str">
         <v>CR</v>
       </c>
       <c r="C4" t="str">
-        <v>501</v>
+        <v>202</v>
       </c>
       <c r="D4" t="str">
-        <v>+961 70 361 683</v>
+        <v>+961 70 108 759</v>
       </c>
       <c r="E4" t="str">
-        <v>today+174d-12m</v>
+        <v>today+181d-24m</v>
       </c>
       <c r="F4" t="str">
-        <v>today+174d</v>
+        <v>today+181d</v>
       </c>
       <c r="G4">
-        <v>1250</v>
+        <v>1000</v>
       </c>
       <c r="H4">
-        <v>1250</v>
+        <v>1000</v>
       </c>
       <c r="I4">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="J4" t="str">
         <v>bank_transfer</v>
@@ -2063,22 +2063,22 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>CR-401-01</v>
+        <v>CR-101-01</v>
       </c>
       <c r="B5" t="str">
         <v>CR</v>
       </c>
       <c r="C5" t="str">
-        <v>401</v>
+        <v>101</v>
       </c>
       <c r="D5" t="str">
-        <v>+961 78 442 534</v>
+        <v>+961 78 258 933</v>
       </c>
       <c r="E5" t="str">
-        <v>today+134d-12m</v>
+        <v>today+258d-12m</v>
       </c>
       <c r="F5" t="str">
-        <v>today+134d</v>
+        <v>today+258d</v>
       </c>
       <c r="G5">
         <v>1125</v>
@@ -2087,7 +2087,7 @@
         <v>1125</v>
       </c>
       <c r="I5">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="J5" t="str">
         <v>cash</v>
@@ -2107,34 +2107,34 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>CR-203-01</v>
+        <v>CR-102-01</v>
       </c>
       <c r="B6" t="str">
         <v>CR</v>
       </c>
       <c r="C6" t="str">
-        <v>203</v>
+        <v>102</v>
       </c>
       <c r="D6" t="str">
-        <v>+961 70 219 593</v>
+        <v>+961 81 751 494</v>
       </c>
       <c r="E6" t="str">
-        <v>today+102d-24m</v>
+        <v>today+268d-24m</v>
       </c>
       <c r="F6" t="str">
-        <v>today+102d</v>
+        <v>today+268d</v>
       </c>
       <c r="G6">
-        <v>775</v>
+        <v>975</v>
       </c>
       <c r="H6">
-        <v>775</v>
+        <v>975</v>
       </c>
       <c r="I6">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="J6" t="str">
-        <v>cash</v>
+        <v>bank_transfer</v>
       </c>
       <c r="K6" t="str">
         <v/>
@@ -2151,34 +2151,34 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>CR-503-01</v>
+        <v>CR-302-01</v>
       </c>
       <c r="B7" t="str">
         <v>CR</v>
       </c>
       <c r="C7" t="str">
-        <v>503</v>
+        <v>302</v>
       </c>
       <c r="D7" t="str">
-        <v>+961 81 284 501</v>
+        <v>+961 79 533 713</v>
       </c>
       <c r="E7" t="str">
-        <v>today+189d-12m</v>
+        <v>today+162d-12m</v>
       </c>
       <c r="F7" t="str">
-        <v>today+189d</v>
+        <v>today+162d</v>
       </c>
       <c r="G7">
-        <v>825</v>
+        <v>1025</v>
       </c>
       <c r="H7">
-        <v>825</v>
+        <v>1025</v>
       </c>
       <c r="I7">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J7" t="str">
-        <v>bank_transfer</v>
+        <v>cheque</v>
       </c>
       <c r="K7" t="str">
         <v/>
@@ -2195,34 +2195,34 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>CR-403-01</v>
+        <v>CR-503-01</v>
       </c>
       <c r="B8" t="str">
         <v>CR</v>
       </c>
       <c r="C8" t="str">
-        <v>403</v>
+        <v>503</v>
       </c>
       <c r="D8" t="str">
-        <v>+961 78 477 783</v>
+        <v>+961 71 801 321</v>
       </c>
       <c r="E8" t="str">
-        <v>today+227d-24m</v>
+        <v>today+189d-12m</v>
       </c>
       <c r="F8" t="str">
-        <v>today+227d</v>
+        <v>today+189d</v>
       </c>
       <c r="G8">
-        <v>800</v>
+        <v>875</v>
       </c>
       <c r="H8">
-        <v>800</v>
+        <v>875</v>
       </c>
       <c r="I8">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="J8" t="str">
-        <v>bank_transfer</v>
+        <v>cash</v>
       </c>
       <c r="K8" t="str">
         <v/>
@@ -2239,31 +2239,31 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>CR-303-01</v>
+        <v>CR-603-01</v>
       </c>
       <c r="B9" t="str">
         <v>CR</v>
       </c>
       <c r="C9" t="str">
-        <v>303</v>
+        <v>603</v>
       </c>
       <c r="D9" t="str">
-        <v>+961 3 478 366</v>
+        <v>+961 78 828 106</v>
       </c>
       <c r="E9" t="str">
-        <v>today+230d-12m</v>
+        <v>today+197d-24m</v>
       </c>
       <c r="F9" t="str">
-        <v>today+230d</v>
+        <v>today+197d</v>
       </c>
       <c r="G9">
-        <v>775</v>
+        <v>850</v>
       </c>
       <c r="H9">
-        <v>775</v>
+        <v>850</v>
       </c>
       <c r="I9">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="J9" t="str">
         <v>bank_transfer</v>
@@ -2283,28 +2283,28 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>CR-602-01</v>
+        <v>CR-401-01</v>
       </c>
       <c r="B10" t="str">
         <v>CR</v>
       </c>
       <c r="C10" t="str">
-        <v>602</v>
+        <v>401</v>
       </c>
       <c r="D10" t="str">
-        <v>+961 78 848 533</v>
+        <v>+961 79 438 693</v>
       </c>
       <c r="E10" t="str">
-        <v>today+162d-12m</v>
+        <v>today+317d-12m</v>
       </c>
       <c r="F10" t="str">
-        <v>today+162d</v>
+        <v>today+317d</v>
       </c>
       <c r="G10">
-        <v>1050</v>
+        <v>1250</v>
       </c>
       <c r="H10">
-        <v>1050</v>
+        <v>1250</v>
       </c>
       <c r="I10">
         <v>17</v>
@@ -2327,34 +2327,34 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>CR-301-01</v>
+        <v>CR-402-01</v>
       </c>
       <c r="B11" t="str">
         <v>CR</v>
       </c>
       <c r="C11" t="str">
-        <v>301</v>
+        <v>402</v>
       </c>
       <c r="D11" t="str">
-        <v>+961 71 801 321</v>
+        <v>+961 78 872 553</v>
       </c>
       <c r="E11" t="str">
-        <v>today+189d-12m</v>
+        <v>today+141d-12m</v>
       </c>
       <c r="F11" t="str">
-        <v>today+189d</v>
+        <v>today+141d</v>
       </c>
       <c r="G11">
-        <v>1200</v>
+        <v>1050</v>
       </c>
       <c r="H11">
-        <v>1200</v>
+        <v>1050</v>
       </c>
       <c r="I11">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J11" t="str">
-        <v>cash</v>
+        <v>bank_transfer</v>
       </c>
       <c r="K11" t="str">
         <v/>
@@ -2371,31 +2371,31 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>CR-101-01</v>
+        <v>CR-502-01</v>
       </c>
       <c r="B12" t="str">
         <v>CR</v>
       </c>
       <c r="C12" t="str">
-        <v>101</v>
+        <v>502</v>
       </c>
       <c r="D12" t="str">
-        <v>+961 78 828 106</v>
+        <v>+961 70 701 949</v>
       </c>
       <c r="E12" t="str">
-        <v>today+197d-24m</v>
+        <v>today+188d-12m</v>
       </c>
       <c r="F12" t="str">
-        <v>today+197d</v>
+        <v>today+188d</v>
       </c>
       <c r="G12">
-        <v>1075</v>
+        <v>1050</v>
       </c>
       <c r="H12">
-        <v>1075</v>
+        <v>1050</v>
       </c>
       <c r="I12">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="J12" t="str">
         <v>bank_transfer</v>
@@ -2415,34 +2415,34 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>CR-202-01</v>
+        <v>CR-403-01</v>
       </c>
       <c r="B13" t="str">
         <v>CR</v>
       </c>
       <c r="C13" t="str">
-        <v>202</v>
+        <v>403</v>
       </c>
       <c r="D13" t="str">
-        <v>+961 71 601 199</v>
+        <v>+961 81 524 789</v>
       </c>
       <c r="E13" t="str">
-        <v>today+270d-12m</v>
+        <v>today+99d-24m</v>
       </c>
       <c r="F13" t="str">
-        <v>today+270d</v>
+        <v>today+99d</v>
       </c>
       <c r="G13">
-        <v>925</v>
+        <v>900</v>
       </c>
       <c r="H13">
-        <v>925</v>
+        <v>900</v>
       </c>
       <c r="I13">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="J13" t="str">
-        <v>bank_transfer</v>
+        <v>cash</v>
       </c>
       <c r="K13" t="str">
         <v/>
@@ -2459,31 +2459,31 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CR-201-01</v>
+        <v>CR-303-01</v>
       </c>
       <c r="B14" t="str">
         <v>CR</v>
       </c>
       <c r="C14" t="str">
-        <v>201</v>
+        <v>303</v>
       </c>
       <c r="D14" t="str">
-        <v>+961 76 851 237</v>
+        <v>+961 70 969 500</v>
       </c>
       <c r="E14" t="str">
-        <v>today+115d-12m</v>
+        <v>today+208d-12m</v>
       </c>
       <c r="F14" t="str">
-        <v>today+115d</v>
+        <v>today+208d</v>
       </c>
       <c r="G14">
-        <v>1200</v>
+        <v>825</v>
       </c>
       <c r="H14">
-        <v>1200</v>
+        <v>825</v>
       </c>
       <c r="I14">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="J14" t="str">
         <v>bank_transfer</v>
@@ -2503,34 +2503,34 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>CR-603-01</v>
+        <v>CR-602-01</v>
       </c>
       <c r="B15" t="str">
         <v>CR</v>
       </c>
       <c r="C15" t="str">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D15" t="str">
-        <v>+961 70 124 242</v>
+        <v>+961 3 800 428</v>
       </c>
       <c r="E15" t="str">
-        <v>today+192d-12m</v>
+        <v>today+120d-12m</v>
       </c>
       <c r="F15" t="str">
-        <v>today+192d</v>
+        <v>today+120d</v>
       </c>
       <c r="G15">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="H15">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="I15">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="J15" t="str">
-        <v>bank_transfer</v>
+        <v>cash</v>
       </c>
       <c r="K15" t="str">
         <v/>
@@ -2590,7 +2590,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>+961 78 442 534</v>
+        <v>+961 70 108 759</v>
       </c>
       <c r="B2" t="str">
         <v>id</v>
@@ -2599,16 +2599,16 @@
         <v>National ID</v>
       </c>
       <c r="D2" t="str">
-        <v>maria-chehab-id.pdf</v>
+        <v>antoine-baydoun-id.pdf</v>
       </c>
       <c r="E2" t="str">
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>today-8y</v>
+        <v>today-5y</v>
       </c>
       <c r="G2" t="str">
-        <v>today+44d</v>
+        <v>today+2y</v>
       </c>
     </row>
   </sheetData>

</xml_diff>